<commit_message>
feat: apply comprehensive QoL transparency updates for skills
apply comprehensive QoL transparency updates for skills, passives,
magic, and items
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/items.xlsx
+++ b/mod_project/data_tables/items.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>A fresh, flaky crescent pastry. Restores 60 HP to one ally.</t>
+          <t>Restore an ally's HP by 60.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>A sweet fruit-topped bakery treat. Restores 250 HP to one ally.</t>
+          <t>Restore an ally's HP by 250.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>A hearty and satisfying bagel meal. Restores 500 HP to one ally.</t>
+          <t>Restore an ally's HP by 500.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>A luxurious bakery treat. Fully restores an ally's HP (9,999 HP).</t>
+          <t>Fully restore an ally's HP (9,999 HP).</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Rich chocolate cake baked to share. Restores 100 HP to all allies.</t>
+          <t>Restore all allies' HP by 100.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -682,9 +682,14 @@
           <t>Restore all allies' HP (medium).</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Restore all allies' HP by 200.</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -712,9 +717,14 @@
           <t>Restore all allies' HP (large).</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Restore all allies' HP by 500.</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -742,9 +752,14 @@
           <t>Sandwich filled with soft, fluffy eggs.</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Fluffy egg sandwich. Restores 10 HP to an ally.</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -772,9 +787,14 @@
           <t>Bread stuffed with yakisoba noodles. Sells out very quickly.</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Noodle-stuffed bread. Restores 20 HP to an ally.</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -802,9 +822,14 @@
           <t>Premium steak sandwich with luxury sauce. Extra deluxe.</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Deluxe steak sandwich. Restores 30 HP to an ally.</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -834,7 +859,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Super spicy curry. Restores 200 HP and boosts physical ATK for 3 turns.</t>
+          <t>Super spicy curry. Restores 150 HP to an ally.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -867,9 +892,14 @@
           <t>Legendary food that's said to make any who eats it fall in love.</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Legendary curry. Restores 1,000 HP to an ally.</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -897,9 +927,14 @@
           <t>Restore an ally's TP (small). The flavor is good as well.</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Restore an ally's TP by 25.</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -927,9 +962,14 @@
           <t>Restore an ally's TP (medium). Fairies love 'em.</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Restore an ally's TP by 50.</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -957,9 +997,14 @@
           <t>Restore an ally's TP (large). Intimidating but delicious.</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Restore an ally's TP by 100.</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -987,9 +1032,14 @@
           <t>Cure one status ailment for an ally. Somewhat bitter.</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Cure one status ailment for an ally.</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -1017,9 +1067,14 @@
           <t>Cure all status ailments for an ally. Sweet to the taste.</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Cure all status ailments for an ally.</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -1047,9 +1102,14 @@
           <t>Revive a fallen ally. Considerably bitter aftertaste.</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Revive a fallen ally with 10% HP.</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -1287,9 +1347,14 @@
           <t>High in nutritional value, it heals HP and TP but is extremely bitter.</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Nutritional tea. Restores 50 HP and 50 TP to an ally.</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9182,9 +9247,14 @@
           <t>A delicious hotpot dish with an addicting smell.</t>
         </is>
       </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Delicious hotpot dish. Restores 150 HP to an ally.</t>
+        </is>
+      </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9242,9 +9312,14 @@
           <t>A slightly disgusting dish made with simmered bear paw.</t>
         </is>
       </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Simmered bear paw dish. Restores 300 HP to an ally.</t>
+        </is>
+      </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14112,9 +14187,14 @@
           <t>Simple hotpot of whale and mizuna.</t>
         </is>
       </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Whale and mizuna hotpot. Restores 400 HP to an ally.</t>
+        </is>
+      </c>
       <c r="G479" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14912,9 +14992,14 @@
           <t>Small candy with a rugged shape.</t>
         </is>
       </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Small rugged candy. Restores 60 HP to an ally.</t>
+        </is>
+      </c>
       <c r="G506" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14942,9 +15027,14 @@
           <t>A larger-scale konpeito.</t>
         </is>
       </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Large-scale konpeito. Restores 120 HP to an ally.</t>
+        </is>
+      </c>
       <c r="G507" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: apply QA audit resolutions for unique skills
apply QA audit resolutions for unique skills, range steps, item wording,
and audit tool
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/items.xlsx
+++ b/mod_project/data_tables/items.xlsx
@@ -754,7 +754,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Fluffy egg sandwich. Restores 10 HP to an ally.</t>
+          <t>Restore an ally's HP by 10.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Noodle-stuffed bread. Restores 20 HP to an ally.</t>
+          <t>Restore an ally's HP by 20.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Deluxe steak sandwich. Restores 30 HP to an ally.</t>
+          <t>Restore an ally's HP by 30.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Super spicy curry. Restores 150 HP to an ally.</t>
+          <t>Restore an ally's HP by 150.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Legendary curry. Restores 1,000 HP to an ally.</t>
+          <t>Restore an ally's HP by 1,000.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Nutritional tea. Restores 50 HP and 50 TP to an ally.</t>
+          <t>Restore an ally's HP by 50 and TP by 50.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>A soothing herbal tincture. Clears overworked vision, curing Blindness.</t>
+          <t>Cure Blindness for an ally.</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -9249,7 +9249,7 @@
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>Delicious hotpot dish. Restores 150 HP to an ally.</t>
+          <t>Restore an ally's HP by 150.</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>Simmered bear paw dish. Restores 300 HP to an ally.</t>
+          <t>Restore an ally's HP by 300.</t>
         </is>
       </c>
       <c r="G314" t="inlineStr">
@@ -14189,7 +14189,7 @@
       </c>
       <c r="F479" t="inlineStr">
         <is>
-          <t>Whale and mizuna hotpot. Restores 400 HP to an ally.</t>
+          <t>Restore an ally's HP by 400.</t>
         </is>
       </c>
       <c r="G479" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="F506" t="inlineStr">
         <is>
-          <t>Small rugged candy. Restores 60 HP to an ally.</t>
+          <t>Restore an ally's HP by 60.</t>
         </is>
       </c>
       <c r="G506" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="F507" t="inlineStr">
         <is>
-          <t>Large-scale konpeito. Restores 120 HP to an ally.</t>
+          <t>Restore an ally's HP by 120.</t>
         </is>
       </c>
       <c r="G507" t="inlineStr">

</xml_diff>

<commit_message>
fix: update Mini Auto-Recovery
update Mini Auto-Recovery, food consumables, and enchant percentage
labels
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/items.xlsx
+++ b/mod_project/data_tables/items.xlsx
@@ -1382,9 +1382,19 @@
           <t>Tea with condensed bitterness. I hear it's an acquired taste...</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Restore an ally's HP by 30 and TP by 40.</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>
@@ -1412,9 +1422,19 @@
           <t>Beard's special bento. A well-balanced meal, and big enough to share.</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Restore all allies' HP by 75 and TP by 25.</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>
@@ -1442,9 +1462,19 @@
           <t>Peggy's eggy milk pudding. It's said to be legendary.</t>
         </is>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Restore an ally's TP by 30. May inflict Sleep.</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>
@@ -1472,9 +1502,19 @@
           <t>Kumaya Mangetsudo's anpan. It's low-calorie, but still delicious.</t>
         </is>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Restore an ally's HP by 20 and TP by 15. May inflict Sleep.</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>
@@ -1502,9 +1542,19 @@
           <t>Mrs. Mary's snack smothered in maple butter.</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Restore an ally's HP by 20 and TP by 15. May inflict Sleep.</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>
@@ -1532,9 +1582,19 @@
           <t>Honey-filled monaka sold at the Kumana Mangetsudo.</t>
         </is>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Restore an ally's TP by 30. May inflict Sleep.</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>
@@ -1647,9 +1707,19 @@
           <t>An exciting new way to cheat death. Courtesy of the Peggy Company.</t>
         </is>
       </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Revive a fallen ally with 100% HP.</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>
@@ -1677,9 +1747,19 @@
           <t>There's a cure for pretty much anything, and there's plenty of it.</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Cure all status ailments for all allies.</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>
@@ -1762,9 +1842,19 @@
           <t>Helpful item to have when push comes to shove.</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Restore all allies' HP by 150.</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>
@@ -1967,9 +2057,19 @@
           <t>A fish cake commonly eaten by ninjas.</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Restore an ally's HP by 100.</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>
@@ -1997,9 +2097,19 @@
           <t>Rock-hard cracker. Not just a snack, but also an emergency ration!</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Restore an ally's HP by 75 and TP by 75.</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>QoL transparency: exact recovery numbers.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: preserve original humor and flavor text across all 388 items
preserve original humor and flavor text across all 388 items with
concise data format
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/items.xlsx
+++ b/mod_project/data_tables/items.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 60.</t>
+          <t>Restore an ally's HP (small) (+60 HP).</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 250.</t>
+          <t>Restore an ally's HP (medium) (+250 HP).</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 500.</t>
+          <t>Restore an ally's HP (large) (+500 HP).</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Fully restore an ally's HP (9,999 HP).</t>
+          <t>Fully restore an ally's HP (Full HP).</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 100.</t>
+          <t>Restore all allies' HP (small) (Party: +100 HP).</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 200.</t>
+          <t>Restore all allies' HP (medium) (Party: +200 HP).</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 500.</t>
+          <t>Restore all allies' HP (large) (Party: +500 HP).</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 10. Cure 1 status ailment.</t>
+          <t>Sandwich filled with soft, fluffy eggs (+10 HP/TP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -829,7 +829,8 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 20. Cure 1 status ailment.</t>
+          <t>Bread stuffed with yakisoba noodles. Sells out very quickly.
+(+20 HP/TP, Cure 1 Ailment)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -869,7 +870,8 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 30. Cure all status ailments.</t>
+          <t>Premium steak sandwich with luxury sauce. Extra deluxe.
+(+30 HP/TP, Cure All Ailments)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -909,7 +911,8 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 150. Cure all status ailments.</t>
+          <t>Super spicy curry that would make even a Maharaja groan.
+(+150 HP/TP, Cure All Ailments)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -949,7 +952,8 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 1,000. Cure all status ailments.</t>
+          <t>Legendary food that's said to make any who eats it fall in love.
+(+1000 HP/TP, Cure All Ailments)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -989,7 +993,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 25.</t>
+          <t>Restore an ally's TP (small). The flavor is good as well (+25 TP).</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1029,7 +1033,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 50.</t>
+          <t>Restore an ally's TP (medium). Fairies love 'em (+50 TP).</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1069,7 +1073,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 100.</t>
+          <t>Restore an ally's TP (large). Intimidating but delicious (+100 TP).</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1109,7 +1113,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Cure 1 status ailment for an ally.</t>
+          <t>Cure one status ailment for an ally. Somewhat bitter (Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1149,7 +1153,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Cure all status ailments for an ally.</t>
+          <t>Cure all status ailments for an ally. Sweet to the taste (Cure All Ailments).</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1189,7 +1193,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Revive a fallen ally with 10% HP.</t>
+          <t>Revive a fallen ally. Considerably bitter aftertaste (Revive 10% HP).</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1229,7 +1233,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Restore all debuffed stats to original levels for an ally.</t>
+          <t>A bell that can restore all debuffed stats to their original levels (Clear Debuffs).</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1269,7 +1273,8 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Cure Shadow Sew and remove skill bind effect for an ally.</t>
+          <t>A charm that cancels Shadow Sew and its skill binding effect.
+(Cure Shadow Sew &amp; Bind)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1309,7 +1314,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Illuminates dark dungeon floors for 10 steps.</t>
+          <t>Lets you light up the dungeon (Light 10 steps).</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1349,7 +1354,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Instantly escape from the dungeon back to base.</t>
+          <t>Lets you escape the dungeon (Escape Dungeon).</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1389,7 +1394,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Permanently grant +3 Skill Points (SP) to an ally.</t>
+          <t>Eat, Skill, Love (+3 SP).</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1429,7 +1434,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Permanently grant +9 Skill Points (SP) to an ally.</t>
+          <t>Even more umami than MSG. Taste the skill points (+9 SP).</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1469,7 +1474,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Permanently grant +9 Skill Points (SP) to an ally.</t>
+          <t>Highly potent skill point extract. A little goes a long way (+9 SP).</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1509,7 +1514,8 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 50 and TP by 20.</t>
+          <t>High in nutritional value, it heals HP and TP but is extremely bitter.
+(+50 HP, +20 TP)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1549,7 +1555,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 30 and TP by 40.</t>
+          <t>Tea with condensed bitterness. I hear it's an acquired taste.. (+30 HP, +40 TP).</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1589,7 +1595,8 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 75 and TP by 25.</t>
+          <t>Beard's special bento. A well-balanced meal, and big enough to share.
+(Party: +75 HP, +25 TP)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1629,7 +1636,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 30. May inflict Sleep (20%).</t>
+          <t>Peggy's eggy milk pudding. It's said to be legendary (+30 TP, 20% Sleep).</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1669,7 +1676,8 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 20. May inflict Sleep (15%).</t>
+          <t>Kumaya Mangetsudo's anpan. It's low-calorie, but still delicious.
+(+20 HP/TP, 15% Sleep)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1709,7 +1717,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 20. May inflict Sleep (15%).</t>
+          <t>Mrs. Mary's snack smothered in maple butter (+20 HP/TP, 15% Sleep).</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1749,7 +1757,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 30. May inflict Sleep (20%).</t>
+          <t>Honey-filled monaka sold at the Kumana Mangetsudo (+30 TP, 20% Sleep).</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1789,7 +1797,8 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Cure all status ailments and stat debuffs for an ally.</t>
+          <t>Consists of Mary Florina's super rich milk collagen. Sorts ailments right out.
+(Cure Ailments &amp; Debuffs)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1864,7 +1873,8 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Nutritious feed for beasts. Restores loyalty and stamina.</t>
+          <t>Beasts love it! The flavor and nutrition balance is just right.
+(Nutritious feed for beasts. Restores loyalty and stamina.)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1904,7 +1914,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Revive a fallen ally with 100% HP.</t>
+          <t>An exciting new way to cheat death. Courtesy of the Peggy Company (Revive 100% HP).</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1944,7 +1954,8 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Cure all status ailments and stat debuffs for an ally.</t>
+          <t>There's a cure for pretty much anything, and there's plenty of it.
+(Cure Ailments &amp; Debuffs)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1979,7 +1990,8 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Deal explosive damage. Inflict Blind (75% chance).</t>
+          <t>A Souffle special. Goes off with a bang that makes you jump.
+(75% Blind, Explosive Dmg)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2019,7 +2031,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Deal 10 fixed damage to an enemy.</t>
+          <t>A Souffle special. Makes a mysterious ticking noise (10 Fixed Dmg).</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2059,7 +2071,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 150.</t>
+          <t>Helpful item to have when push comes to shove (Party: +150 HP).</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2099,7 +2111,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Cure 1 status ailment for an ally.</t>
+          <t>Makes you feel lucky... kinda (Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2139,7 +2151,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Cure all status ailments for an ally.</t>
+          <t>An aged icon that's heard prayers year after year (Cure All Ailments).</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2179,7 +2191,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Restore all debuffed stats to original levels for an ally.</t>
+          <t>A gun shell left by one who gave up their life for revolution (Clear Debuffs).</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2219,7 +2231,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Illuminates dark dungeon floors for 30 steps.</t>
+          <t>A splendidly well-made futuristic metal. It's a bit lumpy. Weird (Light 30 steps).</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2259,7 +2271,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (25% chance).</t>
+          <t>It scrambles your brain, and then you die. No coming back from that (25% Death).</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2334,7 +2346,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100. Restore debuffed stats.</t>
+          <t>A fish cake commonly eaten by ninjas (+100 HP, Clear Debuffs).</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2374,7 +2386,8 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 75. Cure Shadow Sew.</t>
+          <t>Rock-hard cracker. Not just a snack, but also an emergency ration!
+(+75 HP/TP, Cure Shadow Sew)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2594,7 +2607,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Evasion +60%.</t>
+          <t>For those elegant afternoons (+60% EVA).</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2629,7 +2642,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Physical ATK +20%.</t>
+          <t>Everyone has been looking, and we've finally found it! (+20% ATK).</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2809,7 +2822,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (25% chance).</t>
+          <t>When I peeked in, something peeked back... There's someone in there! (25% Death).</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2844,7 +2857,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Physical DEF +40%.</t>
+          <t>A fortunetelling book with a storied history (+40% DEF).</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2884,7 +2897,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Cure Shadow Sew and remove skill bind effect for an ally.</t>
+          <t>Might be usable in traditional medicine... if anything (Cure Shadow Sew &amp; Bind).</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3099,7 +3112,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 175. Physical ATK +75%.</t>
+          <t>Whatever's under all that breading, you can bet it's good and fried (+75% ATK).</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3174,7 +3187,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Inflict Silence (40% chance).</t>
+          <t>Those memories are precious... and painful (40% Silence).</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3284,7 +3297,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Inflict Sleep (50% chance). Physical DEF +75%.</t>
+          <t>A sedative for pregnant women, but there are side effects.. (+75% DEF).</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3394,7 +3407,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Instantly escape from the dungeon back to base.</t>
+          <t>Lets a witch fly free, but takes some practice (Escape Dungeon).</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3434,7 +3447,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Cure all status ailments for an ally.</t>
+          <t>Might's not all that makes right. Money does the trick too (Cure All Ailments).</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3474,7 +3487,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Inflict Silence (50% chance).</t>
+          <t>I must immediately depart on a long, long journey. Don't look for me (50% Silence).</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3509,7 +3522,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Physical ATK +85%. Speed +85%.</t>
+          <t>Compendium of every style made by a master fistfighter (+85% ATK, +85% SPD).</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3549,7 +3562,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 150. Physical ATK +75%.</t>
+          <t>A red feather you receive after donating to a fundraiser (+75% ATK).</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3589,7 +3602,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Inflict Blind (50% chance).</t>
+          <t>Creepy pitch-black rosary (50% Blind).</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3629,7 +3642,8 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Inflict Gray Curse (75% chance).</t>
+          <t>Cursed words from an ex-girlfriend. She's really vile...
+(Inflict Gray Curse (75% chance).)</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3704,7 +3718,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Instantly escape from the dungeon back to base.</t>
+          <t>Down came the rain, but this web did not get washed out (Escape Dungeon).</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -3744,7 +3758,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Inflict Poison (40% chance).</t>
+          <t>One prick with this needle would be disastrous. Handle with care (40% Poison).</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -3784,7 +3798,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Inflict Blind (30% chance).</t>
+          <t>A mirror that reveals the truth... You might not want to look (30% Blind).</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -3859,7 +3873,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 8.</t>
+          <t>It's fantastick! (+8 TP).</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4084,7 +4098,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (90% chance).</t>
+          <t>A disconcerting egg. The face is always screaming (90% Death).</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -4159,7 +4173,8 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Cure 1 status ailment for an ally.</t>
+          <t>Vial of mysterious holy water. Tiny waves are ever-present at the top.
+(Cure 1 Ailment)</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -4199,7 +4214,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 50. Physical ATK +20%.</t>
+          <t>Fried up in an iron pan. A steal at 3 million lira! (+20% ATK).</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -4239,7 +4254,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Inflict Silence (30% chance).</t>
+          <t>There's no wind blowing, yet you can hear its sound. It cries Mary (30% Silence).</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -4349,7 +4364,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Accuracy +80%.</t>
+          <t>Just one drop will refresh constantly overworked eyes (Accuracy +80%.).</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -4389,7 +4404,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Cure all status ailments for an ally.</t>
+          <t>It's not just for petrification anymore! (Cure All Ailments).</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -4429,7 +4444,8 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Illuminates dark dungeon floors for 15 steps.</t>
+          <t>Blowing or splashing water won't put out this fire. We didn't start it.
+(Light 15 steps)</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -4544,7 +4560,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 24.</t>
+          <t>The fruit, sadly, not the special event. Sweet and packed with energy (+24 TP).</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -4584,7 +4600,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 40. May inflict Instant Death (30%).</t>
+          <t>If this is waiting back at the base, you know someone's about to die (+40 TP).</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -4624,7 +4640,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 100 and TP by 40.</t>
+          <t>A pastry for the prosperous. Crumbles on your tongue (Party: +100 HP, +40 TP).</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -4984,7 +5000,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (20% chance).</t>
+          <t>Plan the perfect trip to the world beyond the veil (20% Death).</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -5129,7 +5145,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Evasion +30%.</t>
+          <t>Smooth, sticky lotion for professional use (+30% EVA).</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -5274,7 +5290,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Revive a fallen ally with 35% HP.</t>
+          <t>It makes a nice crunching sound when you bite into it (Revive 35% HP).</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -5314,7 +5330,8 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Cure all status ailments for an ally.</t>
+          <t>A branch only certain people are allowed to pray to. It's twig-sclusive.
+(Cure All Ailments)</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -5384,7 +5401,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Evasion +15%.</t>
+          <t>Sandals that are no longer of any use. Might as well toss 'em (+15% EVA).</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -5534,7 +5551,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Inflict Blind (35% chance).</t>
+          <t>Stone core made when an evil heart has hardened completely (35% Blind).</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -5569,7 +5586,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Physical ATK +50%.</t>
+          <t>Do YOU ever ruin your good cleaver on bone? Finally, there's help! (+50% ATK).</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -5649,7 +5666,8 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>May inflict Curse (50%).</t>
+          <t>Liquor made of crushed fairies. Not guaranteed not to curse you...
+(May inflict Curse (50%).)</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -5689,7 +5707,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Illuminates dark dungeon floors for 5 steps.</t>
+          <t>Lantern that's overused, and somewhat broken (Light 5 steps).</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -5879,7 +5897,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Cure 1 status ailment for an ally.</t>
+          <t>Sparkly and radiant (Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -5989,7 +6007,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 999. 90% risk of Instant Death.</t>
+          <t>Eat this and you may die on the spot... or not at all (+999 TP).</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -6094,7 +6112,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Accuracy +80%.</t>
+          <t>Tonight, I will steal away your heart (Accuracy +80%.).</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -6169,7 +6187,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Cure Freeze for an ally.</t>
+          <t>A support item used by people who can't swim (Cure Freeze).</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -6349,7 +6367,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 95.</t>
+          <t>Fried-up culinary mix of potato... and korpokkur (+95 HP).</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -6389,7 +6407,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 50. Physical ATK +50%.</t>
+          <t>Rice-based liquor aged for more than three years (+50% ATK).</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -6424,7 +6442,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Speed DOWN -60%.</t>
+          <t>For nailing uncooperative ogres to the ground (Speed DOWN -60%.).</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -6624,7 +6642,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 14.</t>
+          <t>A kind of dried food. Rehydrate before cooking (+14 TP).</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -6664,7 +6682,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 60. Evasion +20%.</t>
+          <t>Oil you can rub on a wound in place of salve. If you want (+20% EVA).</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -6744,7 +6762,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Cure Sleep for an ally.</t>
+          <t>Somebody shut it up! (Cure Sleep).</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -6784,7 +6802,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200. May inflict Sleep (75%).</t>
+          <t>Looks like that's a YES (+200 HP, 75% Sleep).</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -6824,7 +6842,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100. Speed +30%.</t>
+          <t>Red and white so you know it's auspicious. Only shaped like a turtle! (+100 HP).</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -6864,7 +6882,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Inflict Poison (75% chance).</t>
+          <t>Huge poisonous spike plucked from a tarasque's back (75% Poison).</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -7014,7 +7032,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Accuracy +30%.</t>
+          <t>Fake version of Alexandrite Cat's Eye (Accuracy +30%.).</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -7124,7 +7142,8 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Instantly teleport back to town/base.</t>
+          <t>Throw it up in the air and maybe you'll warp to a city you've visited before.
+(Instantly teleport back to town/base.)</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -7199,7 +7218,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Inflict Sleep (90% chance).</t>
+          <t>You were forced to buy it at 5x the market price. I could cry (90% Sleep).</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -7239,7 +7258,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Inflict Curse (40% chance).</t>
+          <t>Unfortunately, it's a one-way ticket (Inflict Curse (40% chance).).</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -7279,7 +7298,8 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (60% chance).</t>
+          <t>Apparently it'll send you to another world with just one sip (it's poison).
+(60% Death)</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -7354,7 +7374,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Instantly escape from the dungeon back to base.</t>
+          <t>In illegible letters, it says: I am here (Escape Dungeon).</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -7389,7 +7409,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Evasion +30%.</t>
+          <t>Said to bring its holder happiness (+30% EVA).</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -7429,7 +7449,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Inflict Curse (30% chance).</t>
+          <t>Honestly, just cut me some slack (Inflict Curse (30% chance).).</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -7469,7 +7489,8 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Inflict Silence (30% chance).</t>
+          <t>It says it's lucky. You can't believe everything you read, now can you?
+(30% Silence)</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -7504,7 +7525,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Accuracy +50%.</t>
+          <t>A letter that simply says: You are my fire. My one desire (Accuracy +50%.).</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -7539,7 +7560,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Physical ATK +80%.</t>
+          <t>The prompt asks, who's your personal hero? I wrote, 'Me.' (+80% ATK).</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -7574,7 +7595,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Physical ATK +30%.</t>
+          <t>Tiger scroll filled with innermost secrets of martial arts (+30% ATK).</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -7609,7 +7630,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Physical ATK +50%.</t>
+          <t>The symbol of justice. Who needs bats, anyways? (+50% ATK).</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -7759,7 +7780,8 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 100. May inflict Blind (75%).</t>
+          <t>Holy river water that contains all sorts of extracts. Extracts...
+(+100 TP, 75% Blind)</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
@@ -7944,7 +7966,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Inflict Freeze (40% chance).</t>
+          <t>More of a snow acquaintance. A snowperson at any rate (40% Freeze).</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -8104,7 +8126,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 18.</t>
+          <t>A scent to calm even the most candle-hating heart (+18 TP).</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
@@ -8179,7 +8201,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Cure Shadow Sew for an ally. Restore debuffed stats.</t>
+          <t>Good for massages and hair care and so on (Cure Shadow Sew).</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -8724,7 +8746,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Inflict Blind (50% chance).</t>
+          <t>A sword with a bamboo grip. For some reason, the grip... reeks (50% Blind).</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -8799,7 +8821,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>Inflict Paralysis (50% chance).</t>
+          <t>A giant bloodshot eyeball. At least it's not moving (50% Paralysis).</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -8984,7 +9006,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Inflict Paralysis (35% chance).</t>
+          <t>Despite its not having a head, you swear you've heard it giggle (35% Paralysis).</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -9199,7 +9221,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Inflict Silence (30% chance).</t>
+          <t>Every time you look at it, the people are in different poses (30% Silence).</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -9239,7 +9261,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Inflict Blind (40% chance).</t>
+          <t>A primal scream that resounds through the natural world (40% Blind).</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -9349,7 +9371,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 325.</t>
+          <t>Fried doughball confection. Just one will fill you up (+325 HP).</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
@@ -9424,7 +9446,7 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Cure Freeze for an ally.</t>
+          <t>Low-tech but reliable way to warm up (Cure Freeze).</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -9464,7 +9486,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (30% chance).</t>
+          <t>Not for use indoors. DEFINITELY not for use in a vehicle! (30% Death).</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -9539,7 +9561,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Inflict Blind (15% chance).</t>
+          <t>Used for voodoo curses. Picture your enemy, and give it your all! (15% Blind).</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -9579,7 +9601,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Inflict Poison (20% chance). May inflict Silence (20%).</t>
+          <t>Jelly infused with natural demon... stuff (20% Poison, 20% Silence).</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -9769,7 +9791,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 150. May inflict Freeze (30%).</t>
+          <t>Mist that covers your skin in glossy beads (+150 TP, 30% Freeze).</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -9849,7 +9871,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 75. Restore debuffed stats.</t>
+          <t>A boxful of crackin' chocolate. The ladies love it! (Party: +75 TP, Clear Debuffs).</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -9884,7 +9906,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Speed DOWN -60%.</t>
+          <t>I'd like to think this is the cause for my weight gain.. (Speed DOWN -60%.).</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
@@ -9919,7 +9941,8 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>May inflict Curse (80%).</t>
+          <t>A roiling mass of darkness. And... is that a green lady in there?
+(May inflict Curse (80%).)</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
@@ -10069,7 +10092,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>Inflict Poison (60% chance).</t>
+          <t>It had to be removed due to cavity (60% Poison).</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -10109,7 +10132,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Inflict Paralysis (60% chance).</t>
+          <t>A paralyzing claw that was cut to the quick (60% Paralysis).</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -10189,7 +10212,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 100.</t>
+          <t>No-good apple that tempts women into strife (Party: +100 TP).</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -10334,7 +10357,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 50. Physical ATK +40%.</t>
+          <t>Fruit goes in the dragon. This stuff comes out. Don't ask (+40% ATK).</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
@@ -10409,7 +10432,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Inflict Sleep (20% chance).</t>
+          <t>Used by busy mommy dragons to keep their babies quiet (20% Sleep).</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
@@ -10449,7 +10472,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Inflict Sleep (40% chance).</t>
+          <t>Tough enough to survive in a mouth full of dragon baby teeth (40% Sleep).</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
@@ -10519,7 +10542,7 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>Evasion +30%.</t>
+          <t>A strange substance that feels like nothingness when you touch it (+30% EVA).</t>
         </is>
       </c>
       <c r="G267" t="inlineStr">
@@ -10559,7 +10582,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200. May inflict Sleep (90%).</t>
+          <t>Not for napping in. For hiding people taking naps (+200 HP, 90% Sleep).</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -10599,7 +10622,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Inflict Paralysis (15% chance).</t>
+          <t>A mask that is just gold in color. Not all that glitters is gold (15% Paralysis).</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
@@ -10669,7 +10692,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>Speed +25%.</t>
+          <t>Makes you feel somewhat quicker (Speed +25%.).</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
@@ -10709,7 +10732,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (60% chance).</t>
+          <t>Goodnight forever (60% Death).</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
@@ -10859,7 +10882,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (40% chance).</t>
+          <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! (40% Death).</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
@@ -10899,7 +10922,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (80% chance).</t>
+          <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! #2 (80% Death).</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -10939,7 +10962,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (95% chance).</t>
+          <t>A nice little rowboat. Cruise the river separating life and death (95% Death).</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -10979,7 +11002,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 35. May inflict Sleep (25%).</t>
+          <t>Sweet mint immortali-tea. More relaxing than relaxation itself (+35 TP, 25% Sleep).</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -11019,7 +11042,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Inflict Paralysis (30% chance). May inflict Sleep (30%).</t>
+          <t>So much jealousy, it's visible to the naked eye (30% Paralysis, 30% Sleep).</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
@@ -11059,7 +11082,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>Revive a fallen ally with 15% HP.</t>
+          <t>You'll come back to life. No guarantees about how (Revive 15% HP).</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
@@ -11099,7 +11122,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 60. May inflict Blind (25%).</t>
+          <t>Bun that gives off the taste of the afterlife (+60 HP, 25% Blind).</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
@@ -11174,7 +11197,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>Inflict Curse (20% chance).</t>
+          <t>I really hope my photo's not on there (Inflict Curse (20% chance).).</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
@@ -11249,7 +11272,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>Inflict Paralysis (50% chance).</t>
+          <t>You'll want to stay away from the water this came from (50% Paralysis).</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
@@ -11469,7 +11492,7 @@
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>Inflict Silence (40% chance).</t>
+          <t>Just ignore them (40% Silence).</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
@@ -11509,7 +11532,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>Inflict Blind (60% chance).</t>
+          <t>Disembodied wrist. Scurries all over the floor like a cleaning robot (60% Blind).</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -11544,7 +11567,7 @@
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Speed +40%.</t>
+          <t>Why let it expire it when you die? This license is forever (Speed +40%.).</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -11579,7 +11602,7 @@
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>Speed +60%.</t>
+          <t>Forgeries are more common than the genuine article (Speed +60%.).</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
@@ -11614,7 +11637,7 @@
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>Speed +80%. Evasion +60%.</t>
+          <t>Raise your clock rate for a limited time (+60% EVA).</t>
         </is>
       </c>
       <c r="G296" t="inlineStr">
@@ -11654,7 +11677,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 20. Cure 1 status ailment.</t>
+          <t>Careful there, mate. That's not chocolate (+20 TP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
@@ -11694,7 +11717,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 12. May inflict Freeze (20%).</t>
+          <t>Ice cream in a peach-shaped container (+12 TP, 20% Freeze).</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
@@ -11734,7 +11757,7 @@
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 24. May inflict Sleep (20%).</t>
+          <t>Sweet mixed drink popular with the ladies (+24 TP, 20% Sleep).</t>
         </is>
       </c>
       <c r="G299" t="inlineStr">
@@ -11774,7 +11797,7 @@
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 36. Cure 1 status ailment.</t>
+          <t>Peach-shaped bun eaten in times of celebration (+36 TP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G300" t="inlineStr">
@@ -11814,7 +11837,7 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 30.</t>
+          <t>Not actually persimmon seeds. More a seed-shaped rice snack (+30 HP).</t>
         </is>
       </c>
       <c r="G301" t="inlineStr">
@@ -11854,7 +11877,8 @@
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 15. Cure 1 status ailment.</t>
+          <t>Sweet persimmons fumigated with sulfur for preservation. Tasty.
+(+15 TP, Cure 1 Ailment)</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
@@ -11929,7 +11953,8 @@
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 130. Cure Shadow Sew.</t>
+          <t>Sushi wrapped in persimmon leaves. Don't eat the leaves, kiddo.
+(Party: +130 HP, Cure Shadow Sew)</t>
         </is>
       </c>
       <c r="G304" t="inlineStr">
@@ -11969,7 +11994,8 @@
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 600. Cure Freeze.</t>
+          <t>Stew of bear-meat citatap with pukusakina and plenty of veggies.
+(Party: +600 HP, Cure Freeze)</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
@@ -12009,7 +12035,7 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200. Cure Freeze.</t>
+          <t>Bear soup that warms up your body (+200 HP, Cure Freeze).</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
@@ -12049,7 +12075,7 @@
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 300.</t>
+          <t>Add some rice at the end to make porridge! (Party: +300 HP).</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
@@ -12089,7 +12115,7 @@
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 20. Cure 1 status ailment.</t>
+          <t>Healthy and delicious chicken meatballs (+20 TP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G308" t="inlineStr">
@@ -12129,7 +12155,7 @@
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 320.</t>
+          <t>Enjoy the flavor of the meat! Salt, not sauce! (+320 HP).</t>
         </is>
       </c>
       <c r="G309" t="inlineStr">
@@ -12169,7 +12195,8 @@
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 240. Restore debuffed stats.</t>
+          <t>Piping hot fried chicken. Ask before you add lemon juice, just to be safe.
+(+240 HP, Clear Debuffs)</t>
         </is>
       </c>
       <c r="G310" t="inlineStr">
@@ -12209,7 +12236,7 @@
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 180.</t>
+          <t>Perfect for diets. Though... isn't raw chicken dangerous? (+180 HP).</t>
         </is>
       </c>
       <c r="G311" t="inlineStr">
@@ -12249,7 +12276,7 @@
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 150.</t>
+          <t>A delicious hotpot dish with an addicting smell (Party: +150 HP).</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
@@ -12289,7 +12316,7 @@
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200.</t>
+          <t>Lamb dish with heavy garlic flavor (+200 HP).</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
@@ -12329,7 +12356,7 @@
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 300. Cure all status ailments.</t>
+          <t>A slightly disgusting dish made with simmered bear paw (+300 TP, Cure All Ailments).</t>
         </is>
       </c>
       <c r="G314" t="inlineStr">
@@ -12369,7 +12396,7 @@
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200.</t>
+          <t>Luxury lamb dish with absolutely no bad odor (+200 HP).</t>
         </is>
       </c>
       <c r="G315" t="inlineStr">
@@ -12409,7 +12436,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 50. Evasion +100%.</t>
+          <t>Fried lamb meatballs with strong coriander scent (+100% EVA).</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
@@ -12449,7 +12476,7 @@
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 300. Cure 1 status ailment.</t>
+          <t>Lunch set with bird meat and bear meat mixed together (+300 HP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G317" t="inlineStr">
@@ -12484,7 +12511,7 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>Evasion +80%.</t>
+          <t>Brave penguins gave their lives to bring you fuel and soap (+80% EVA).</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
@@ -12524,7 +12551,7 @@
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100.</t>
+          <t>Drink made by mixing cola and strawberries together (+100 HP).</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
@@ -12564,7 +12591,7 @@
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200. Cure Sleep.</t>
+          <t>Feel refreshed by the mint's cold and transcendent stimulation (+200 HP, Cure Sleep).</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
@@ -12604,7 +12631,7 @@
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 275.</t>
+          <t>Frozen danish with a penguin mark on it (+275 HP).</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
@@ -12644,7 +12671,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 400.</t>
+          <t>Ice cream from the past with a nostalgic texture (+400 HP).</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
@@ -12684,7 +12711,7 @@
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 30.</t>
+          <t>Salmon buried in snow to be preserved by the cold (+30 TP).</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
@@ -12724,7 +12751,7 @@
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 75.</t>
+          <t>All-natural, of course. Gluten-free, too! (+75 TP).</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
@@ -12939,7 +12966,7 @@
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>Cure Shadow Sew and remove skill bind effect for an ally.</t>
+          <t>Oil that reeks of sheep (Cure Shadow Sew &amp; Bind).</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
@@ -13014,7 +13041,7 @@
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>Inflict Poison (5% chance).</t>
+          <t>Supplement with a pungently strange odor (5% Poison).</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
@@ -13054,7 +13081,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>Inflict Blind (10% chance).</t>
+          <t>Sketchy in over seven ways. Get it? Like seven colors of the rainbow! (10% Blind).</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
@@ -13129,7 +13156,7 @@
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100.</t>
+          <t>Fun, colorful rice dumplings on a skewer (+100 HP).</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
@@ -13169,7 +13196,7 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200. Cure 1 status ailment.</t>
+          <t>Rice dumplings glazed in sweet soy (+200 HP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
@@ -13209,7 +13236,7 @@
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 180.</t>
+          <t>Three delicious aspects of the dumpling, together on one skewer (Party: +180 HP).</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
@@ -13249,7 +13276,7 @@
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 180.</t>
+          <t>Freshly cut horse-meat sashimi (+180 HP/TP).</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
@@ -13289,7 +13316,7 @@
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 360. Physical DEF +75%.</t>
+          <t>Aged, well-smoked horse meat. An exquisite dish (+75% DEF).</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
@@ -13329,7 +13356,7 @@
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 2,000.</t>
+          <t>Raw meat cut fine and called a steak. Consume with caution (+2000 HP/TP).</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
@@ -13369,7 +13396,7 @@
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 120.</t>
+          <t>A homemade rice ball made this morning (+120 HP).</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
@@ -13409,7 +13436,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 280.</t>
+          <t>A salmon-filled rice ball that required a lot of effort (+280 HP).</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -13449,7 +13476,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 380.</t>
+          <t>A rice ball stuffed with sour pickled plums (+380 HP).</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
@@ -13489,7 +13516,7 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 420.</t>
+          <t>A warm rice ball, pan-grilled with soy sauce (+420 HP).</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -13529,7 +13556,7 @@
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 515.</t>
+          <t>Glutinous steamed rice dish with big pieces of chestnut (+515 HP).</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
@@ -13569,7 +13596,7 @@
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 105.</t>
+          <t>Chewy on the outside, moist on the inside (+105 HP).</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
@@ -13609,7 +13636,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 135. Accuracy +30%.</t>
+          <t>Seashell-shaped snack. Sally sells them by the seashore (+135 HP).</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -13649,7 +13676,8 @@
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 165. Restore debuffed stats.</t>
+          <t>Solidified syrup and dry fruit. A hard candy for hard men.
+(Party: +165 HP, Clear Debuffs)</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
@@ -13689,7 +13717,8 @@
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 250 and TP by 25.</t>
+          <t>A cake with a figurine in it. Whoever finds the little feller gets to be king.
+(Party: +250 HP, +25 TP)</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
@@ -13729,7 +13758,7 @@
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 30.</t>
+          <t>Not everyone who eats muffins is in the mafia. The muffia? Hyuk hyuk (+30 HP/TP).</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
@@ -13769,7 +13798,7 @@
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 50. Accuracy +50%.</t>
+          <t>Off the shelf or the classy kind? They're really not that different (+50 HP).</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
@@ -13809,7 +13838,7 @@
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 115.</t>
+          <t>Party pastry constructed of fruits, custard, and jelly (Party: +115 TP).</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
@@ -13849,7 +13878,7 @@
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 55.</t>
+          <t>A cookie cut into a simple shape. Ooh, looks like a star! (Party: +55 HP).</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
@@ -13889,7 +13918,7 @@
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 160.</t>
+          <t>A cookie cut into a somewhat complex shape. Ooh, looks like a cow! (Party: +160 HP).</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
@@ -13929,7 +13958,7 @@
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 200.</t>
+          <t>A cookie cut into a highly complex shape. Ooh, looks like Japan! (Party: +200 HP).</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
@@ -13969,7 +13998,7 @@
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 75.</t>
+          <t>Old-fashioned rice cracker covered in soy sauce (+75 HP).</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
@@ -14009,7 +14038,7 @@
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 120.</t>
+          <t>Rice cracker covered in plenty of cayenne powder (+120 HP).</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
@@ -14049,7 +14078,7 @@
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 240.</t>
+          <t>Just a cracker with tasty sauce, but dang, that's tasty (+240 HP).</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -14089,7 +14118,7 @@
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 300.</t>
+          <t>Pre-chewed for convenience. Yum! (+300 HP).</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -14129,7 +14158,7 @@
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100.</t>
+          <t>Dried food with a very particular mouthfeel (+100 HP).</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -14169,7 +14198,7 @@
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 120. May inflict Silence (90%).</t>
+          <t>Extremely smelly and rotten tofu (+120 HP, 90% Silence).</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -14279,7 +14308,7 @@
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 10.</t>
+          <t>Candy that makes your mouth all sticky (+10 TP).</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
@@ -14319,7 +14348,7 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 31. Cure 1 status ailment.</t>
+          <t>Colorful candy that is kneaded with two sticks (+31 TP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
@@ -14359,7 +14388,7 @@
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 46. Cure 1 status ailment.</t>
+          <t>An amber candy (+46 TP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
@@ -14399,7 +14428,7 @@
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 75. Cure 1 status ailment.</t>
+          <t>Intensely sweet sugar candy (+75 TP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
@@ -14439,7 +14468,7 @@
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 150. Accuracy +75%.</t>
+          <t>Eat a long candy, live a long life. It's just math (+150 TP).</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
@@ -14479,7 +14508,7 @@
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>Restore all allies' HP and TP by 666.</t>
+          <t>An extremely rare, top-notch candy from the demon world (Party: +666 HP/TP).</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
@@ -14519,7 +14548,7 @@
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 80. Physical ATK +35%.</t>
+          <t>Meatball patty with conspicuous chunks of onion (+35% ATK).</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
@@ -14559,7 +14588,7 @@
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 300. Physical ATK +75%.</t>
+          <t>Sunny-side up egg on a patty. When to break the yolk...? (+75% ATK).</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
@@ -14594,7 +14623,7 @@
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>Speed +25%.</t>
+          <t>The carbonation feels good as it slides down your throat (Speed +25%.).</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
@@ -14629,7 +14658,7 @@
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>Physical DEF +25%.</t>
+          <t>It's sweet and spicy... What evil genius came up with this?? (+25% DEF).</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
@@ -14664,7 +14693,7 @@
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>Speed +50%. Physical DEF +50%.</t>
+          <t>Hard to understand the point. Unbearably hot (+50% DEF).</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
@@ -14704,7 +14733,7 @@
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200.</t>
+          <t>Wafer sandwich, fully-packed with red beans (+200 HP).</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
@@ -14744,7 +14773,7 @@
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>Inflict Instant Death (95% chance).</t>
+          <t>An ominous monaka in the shape of a coffin (95% Death).</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
@@ -14784,7 +14813,7 @@
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 400. Accuracy +75%.</t>
+          <t>Sesame, white bean paste, and... red bean paste! (+400 HP).</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
@@ -14824,7 +14853,7 @@
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 75.</t>
+          <t>A tiny, yet expensive, pastry (+75 HP).</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
@@ -14864,7 +14893,7 @@
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 150. Accuracy +75%.</t>
+          <t>Bright macarons with an assortment of colors (+150 HP).</t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
@@ -14904,7 +14933,7 @@
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 50. Physical DEF +75%.</t>
+          <t>Cookies for your iron abs (+75% DEF).</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
@@ -14944,7 +14973,7 @@
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100. Physical ATK +50%.</t>
+          <t>Cake for your swole six-pack (+50% ATK).</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
@@ -14984,7 +15013,7 @@
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 300.</t>
+          <t>Staple food on Planet Muscle. Go from ripped to jacked (+300 HP).</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
@@ -15024,7 +15053,7 @@
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 55. May inflict Sleep (10%).</t>
+          <t>Apple drink. Sweet, spiked, or sparkling (+55 TP, 10% Sleep).</t>
         </is>
       </c>
       <c r="G383" t="inlineStr">
@@ -15064,7 +15093,7 @@
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 74. May inflict Sleep (25%).</t>
+          <t>Mellow, rich, and just the right amount of bitter (+74 TP, 25% Sleep).</t>
         </is>
       </c>
       <c r="G384" t="inlineStr">
@@ -15104,7 +15133,7 @@
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 140. May inflict Sleep (35%).</t>
+          <t>Sultry spirit. The perfect apertif (+140 TP, 35% Sleep).</t>
         </is>
       </c>
       <c r="G385" t="inlineStr">
@@ -15144,7 +15173,7 @@
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 999. May inflict Sleep (45%).</t>
+          <t>The oil of conversation. The philosophic wine (+999 TP, 45% Sleep).</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
@@ -15184,7 +15213,7 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 20. May inflict Silence (40%).</t>
+          <t>You know you should stop but you just can't kelp yourself (+20 TP, 40% Silence).</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
@@ -15224,7 +15253,7 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 30. May inflict Silence (60%).</t>
+          <t>Sandfish simmered in sugar and soy sauce (+30 TP, 60% Silence).</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
@@ -15264,7 +15293,8 @@
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 40. May inflict Silence (60%).</t>
+          <t>If you get served this without a warning, you're the butt of a joke.
+(+40 TP, 60% Silence)</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
@@ -15304,7 +15334,7 @@
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 50. May inflict Silence (60%).</t>
+          <t>Bad looks and worse texture but weirdly addictive (+50 TP, 60% Silence).</t>
         </is>
       </c>
       <c r="G390" t="inlineStr">
@@ -15344,7 +15374,8 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 160.</t>
+          <t>Flatten an octopus and this is what you get. There's plenty to go around.
+(Party: +160 HP)</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -15384,7 +15415,7 @@
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 400. Physical ATK +50%.</t>
+          <t>Rice with big ol' chunks of tentacle (+50% ATK).</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
@@ -15424,7 +15455,7 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 125.</t>
+          <t>Completely, utterly, absolutely flavorless (+125 TP).</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
@@ -15464,7 +15495,7 @@
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 200.</t>
+          <t>Apparently the primary source of sustenance for one particular race (+200 HP/TP).</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
@@ -15504,7 +15535,7 @@
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 20.</t>
+          <t>A foreign snack smothered in syrupy goodness (+20 TP).</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
@@ -15544,7 +15575,7 @@
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 44.</t>
+          <t>Tastes... sweet. Nothing but sweet. Not to be confused with balaclava (+44 TP).</t>
         </is>
       </c>
       <c r="G396" t="inlineStr">
@@ -15584,7 +15615,7 @@
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 72.</t>
+          <t>A runny, sugary snack. The calorie content must be through the roof (+72 TP).</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
@@ -15624,7 +15655,7 @@
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 98. Accuracy +50%.</t>
+          <t>Spiral sweet soaked in sugary syrup (+98 TP).</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
@@ -15664,7 +15695,7 @@
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 25.</t>
+          <t>Rather bland-tasting. A wholly disappointing dish (+25 TP).</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
@@ -15704,7 +15735,7 @@
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 60. Cure 1 status ailment.</t>
+          <t>Fluffy food with a mesh pattern (+60 TP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G400" t="inlineStr">
@@ -15744,7 +15775,7 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 50. Restore debuffed stats.</t>
+          <t>Waffle made with rice flour. Comes out mochi-ish (+50 TP, Clear Debuffs).</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
@@ -15784,7 +15815,7 @@
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 85. Cure all status ailments.</t>
+          <t>A sweet waffle with syrup mixed into the batter (+85 TP, Cure All Ailments).</t>
         </is>
       </c>
       <c r="G402" t="inlineStr">
@@ -15824,7 +15855,7 @@
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 160. Cure all status ailments.</t>
+          <t>Luxury pancakes like you only get at overpriced hotels (+160 TP, Cure All Ailments).</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
@@ -15864,7 +15895,7 @@
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 30.</t>
+          <t>Which end do you eat it from? It's a matter of scholarly debate (+30 TP).</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
@@ -15904,7 +15935,7 @@
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 58.</t>
+          <t>Tough rye bread that poses a challenge for seniors with weak teeth (+58 HP).</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -15944,7 +15975,7 @@
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 400.</t>
+          <t>Red bean bun baked with fine gold wheat. Diabetics should avoid it (+400 HP).</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
@@ -15984,7 +16015,7 @@
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 75.</t>
+          <t>Snack made by frying sliced potatoes. Also known as crisps (+75 HP).</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
@@ -16024,7 +16055,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 120. Physical DEF +75%.</t>
+          <t>Potato chips covered with habanero powder (+75% DEF).</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -16059,7 +16090,7 @@
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>Physical ATK +40%. May inflict Blind (70%).</t>
+          <t>Potato chips that'll blow your top (+40% ATK).</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
@@ -16099,7 +16130,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 20.</t>
+          <t>Nana always has one or two in her bag. It's the law (+20 HP).</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
@@ -16139,7 +16170,7 @@
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 70.</t>
+          <t>Invokes the undeniable urge to rap. You'll be a real Kandy-e West (+70 HP).</t>
         </is>
       </c>
       <c r="G411" t="inlineStr">
@@ -16179,7 +16210,7 @@
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 150.</t>
+          <t>A high-class rusk coated in white chocolate. Mindblowingly delicious (+150 HP).</t>
         </is>
       </c>
       <c r="G412" t="inlineStr">
@@ -16219,7 +16250,7 @@
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 300. May inflict Silence (30%).</t>
+          <t>A candy so sweet it will cause your brain to melt (+300 HP, 30% Silence).</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
@@ -16259,7 +16290,7 @@
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t>Inflict Paralysis (25% chance).</t>
+          <t>So spicy it makes your eyes hurt (25% Paralysis).</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
@@ -16299,7 +16330,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 50. Cure Freeze.</t>
+          <t>Eat it and you'll sweat from every orifice you've got (+50 HP, Cure Freeze).</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
@@ -16339,7 +16370,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 75. May inflict Paralysis (15%).</t>
+          <t>First-timers will lose consciousness due to the spice (+75 HP/TP, 15% Paralysis).</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
@@ -16379,7 +16410,8 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 400. May inflict Silence (80%).</t>
+          <t>So spicy, it's out of this world. Just one phone call and they'll deliver.
+(+400 HP, 80% Silence)</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
@@ -16419,7 +16451,7 @@
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 90.</t>
+          <t>Fresh, warm donut (+90 HP).</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
@@ -16459,7 +16491,7 @@
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200.</t>
+          <t>Donut with red bean paste on the inside, sugar coating on the outside (+200 HP).</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">
@@ -16499,7 +16531,7 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 25.</t>
+          <t>Sweet and tasty almond-flavored tofu (+25 TP).</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
@@ -16539,7 +16571,7 @@
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 100. Physical DEF +50%.</t>
+          <t>Exquisite and jiggly almond-flavored tofu (+50% DEF).</t>
         </is>
       </c>
       <c r="G421" t="inlineStr">
@@ -16579,7 +16611,7 @@
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 130.</t>
+          <t>A fish-shaped cake filled with red beans from head to tail (+130 HP).</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
@@ -16619,7 +16651,7 @@
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200 and TP by 40.</t>
+          <t>Taiyaki with matcha mixed into the batter. Looks a little gross (+200 HP, +40 TP).</t>
         </is>
       </c>
       <c r="G423" t="inlineStr">
@@ -16659,7 +16691,7 @@
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 40.</t>
+          <t>The shrooms of the hills despise the coddled city bamboo shoots (+40 TP).</t>
         </is>
       </c>
       <c r="G424" t="inlineStr">
@@ -16699,7 +16731,7 @@
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 40. Restore debuffed stats.</t>
+          <t>Safe, cheap, and tropical (+40 TP, Clear Debuffs).</t>
         </is>
       </c>
       <c r="G425" t="inlineStr">
@@ -16809,7 +16841,7 @@
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 40.</t>
+          <t>The perfect dessert for a hot day (+40 TP).</t>
         </is>
       </c>
       <c r="G428" t="inlineStr">
@@ -16849,7 +16881,7 @@
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 75.</t>
+          <t>Shaved ice with some joyous rice-flour dumplings (+75 TP).</t>
         </is>
       </c>
       <c r="G429" t="inlineStr">
@@ -16889,7 +16921,7 @@
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 160. Cure Freeze.</t>
+          <t>Refrigerated agar with added beans and fruits (+160 TP, Cure Freeze).</t>
         </is>
       </c>
       <c r="G430" t="inlineStr">
@@ -16929,7 +16961,7 @@
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 105.</t>
+          <t>A grab bag of vegetables! Rabbit food. Hooray (+105 HP).</t>
         </is>
       </c>
       <c r="G431" t="inlineStr">
@@ -16969,7 +17001,7 @@
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 45.</t>
+          <t>Salad showered with colorful flower petals (+45 TP).</t>
         </is>
       </c>
       <c r="G432" t="inlineStr">
@@ -17009,7 +17041,7 @@
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 135.</t>
+          <t>An assortment of sweet fruits (+135 TP).</t>
         </is>
       </c>
       <c r="G433" t="inlineStr">
@@ -17049,7 +17081,7 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 150.</t>
+          <t>Opulent Chinese vegetable dish. Contains no meat. For some reason (+150 TP).</t>
         </is>
       </c>
       <c r="G434" t="inlineStr">
@@ -17089,7 +17121,8 @@
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100. Cure 1 status ailment.</t>
+          <t>This sticky pudding is speckled with raisins. It's just pudding. Honestly.
+(+100 HP, Cure 1 Ailment)</t>
         </is>
       </c>
       <c r="G435" t="inlineStr">
@@ -17129,7 +17162,7 @@
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 280. Cure 1 status ailment.</t>
+          <t>A cakey treat filled with delicious red bean paste (+280 HP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G436" t="inlineStr">
@@ -17169,7 +17202,7 @@
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 125.</t>
+          <t>Ol' reliable. You can't go wrong with bean paste (+125 TP).</t>
         </is>
       </c>
       <c r="G437" t="inlineStr">
@@ -17209,7 +17242,7 @@
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 10.</t>
+          <t>Soup made wholly out of leftovers. Liver and let die! (Party: +10 TP).</t>
         </is>
       </c>
       <c r="G438" t="inlineStr">
@@ -17249,7 +17282,7 @@
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 25.</t>
+          <t>The unagi's not necessarily good, but the sauce is (Party: +25 TP).</t>
         </is>
       </c>
       <c r="G439" t="inlineStr">
@@ -17289,7 +17322,7 @@
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 50.</t>
+          <t>Dead eels on rice. It's terrible, you wouldn't want any (Party: +50 TP).</t>
         </is>
       </c>
       <c r="G440" t="inlineStr">
@@ -17329,7 +17362,8 @@
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 30. May inflict Silence (50%).</t>
+          <t>Sushi roll containing sticky, smelly, fermented soybeans. Yum...?
+(+30 HP/TP, 50% Silence)</t>
         </is>
       </c>
       <c r="G441" t="inlineStr">
@@ -17369,7 +17403,7 @@
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 60. May inflict Silence (60%).</t>
+          <t>You must be mindful of your surroundings when eating this (+60 HP/TP, 60% Silence).</t>
         </is>
       </c>
       <c r="G442" t="inlineStr">
@@ -17409,7 +17443,7 @@
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 100. May inflict Silence (70%).</t>
+          <t>Extremely smelly... but somehow delicious (+100 HP/TP, 70% Silence).</t>
         </is>
       </c>
       <c r="G443" t="inlineStr">
@@ -17449,7 +17483,7 @@
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 40. Physical DEF +30%.</t>
+          <t>Silky-smooth little fish, rich in calcium (+30% DEF).</t>
         </is>
       </c>
       <c r="G444" t="inlineStr">
@@ -17489,7 +17523,7 @@
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100. May inflict Blind (40%).</t>
+          <t>Somewhat grotesque when the fish has the face of a man (+100 HP, 40% Blind).</t>
         </is>
       </c>
       <c r="G445" t="inlineStr">
@@ -17529,7 +17563,7 @@
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 120. Physical DEF +60%.</t>
+          <t>Well dried bonito flakes (+60% DEF).</t>
         </is>
       </c>
       <c r="G446" t="inlineStr">
@@ -17569,7 +17603,7 @@
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200. Physical DEF +80%.</t>
+          <t>Bonito so dry it's a blunt weapon. The world's hardest food (+80% DEF).</t>
         </is>
       </c>
       <c r="G447" t="inlineStr">
@@ -17609,7 +17643,7 @@
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 18.</t>
+          <t>Cucumber sushi. The kappa's favorite (+18 TP).</t>
         </is>
       </c>
       <c r="G448" t="inlineStr">
@@ -17649,7 +17683,7 @@
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 50 and TP by 10.</t>
+          <t>A simple but deep sushi. Make this your last order to look cultured (+50 HP, +10 TP).</t>
         </is>
       </c>
       <c r="G449" t="inlineStr">
@@ -17689,7 +17723,8 @@
       </c>
       <c r="F450" t="inlineStr">
         <is>
-          <t>Cure all status ailments for an ally.</t>
+          <t>Bitter jelly allegedly good for the skin. Not so great for the tortoise.
+(Cure All Ailments)</t>
         </is>
       </c>
       <c r="G450" t="inlineStr">
@@ -17729,7 +17764,7 @@
       </c>
       <c r="F451" t="inlineStr">
         <is>
-          <t>Cure all status ailments for an ally.</t>
+          <t>Genuine, honest, real turtle soup! Would I lie to you? (Cure All Ailments).</t>
         </is>
       </c>
       <c r="G451" t="inlineStr">
@@ -17769,7 +17804,8 @@
       </c>
       <c r="F452" t="inlineStr">
         <is>
-          <t>Cure all status ailments for an ally. Restore TP by 125.</t>
+          <t>Made in an earthenware pot at high temperature. Delicious but steep.
+(+125 TP, Cure All Ailments)</t>
         </is>
       </c>
       <c r="G452" t="inlineStr">
@@ -17809,7 +17845,7 @@
       </c>
       <c r="F453" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100.</t>
+          <t>Regular size, smothered with sauce please! (+100 HP).</t>
         </is>
       </c>
       <c r="G453" t="inlineStr">
@@ -17849,7 +17885,7 @@
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 150. Physical ATK +50%.</t>
+          <t>Bento with only meat and rice. Get those veggies out of here! (+50% ATK).</t>
         </is>
       </c>
       <c r="G454" t="inlineStr">
@@ -17889,7 +17925,7 @@
       </c>
       <c r="F455" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200. Physical ATK +70%.</t>
+          <t>Sukiyaki bento with super luxurious wagyu included (+70% ATK).</t>
         </is>
       </c>
       <c r="G455" t="inlineStr">
@@ -17929,7 +17965,7 @@
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 400. Physical ATK +90%.</t>
+          <t>Steak bento so delicious it'll make you dizzy (+90% ATK).</t>
         </is>
       </c>
       <c r="G456" t="inlineStr">
@@ -17969,7 +18005,7 @@
       </c>
       <c r="F457" t="inlineStr">
         <is>
-          <t>Inflict Poison (60% chance).</t>
+          <t>A liquid formed from the drool of the elusive nuko (60% Poison).</t>
         </is>
       </c>
       <c r="G457" t="inlineStr">
@@ -18009,7 +18045,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 30.</t>
+          <t>Sake with silver vine for added energy. Do it for the vine! (+30 TP).</t>
         </is>
       </c>
       <c r="G458" t="inlineStr">
@@ -18049,7 +18085,7 @@
       </c>
       <c r="F459" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 60.</t>
+          <t>Try to point out that it's yellow, and a rep will appear to call it gold (+60 TP).</t>
         </is>
       </c>
       <c r="G459" t="inlineStr">
@@ -18089,7 +18125,7 @@
       </c>
       <c r="F460" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 75. 20% risk of Instant Death.</t>
+          <t>Don't drink too much if you like your brain cells (+75 TP).</t>
         </is>
       </c>
       <c r="G460" t="inlineStr">
@@ -18129,7 +18165,7 @@
       </c>
       <c r="F461" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 80.</t>
+          <t>It takes a lot of effort to make (+80 HP).</t>
         </is>
       </c>
       <c r="G461" t="inlineStr">
@@ -18169,7 +18205,8 @@
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 135. Cure Shadow Sew.</t>
+          <t>Cheap and delicious. Sometimes filled with strawberry or pudding.
+(+135 HP, Cure Shadow Sew)</t>
         </is>
       </c>
       <c r="G462" t="inlineStr">
@@ -18209,7 +18246,7 @@
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 225. Cure 1 status ailment.</t>
+          <t>Mochi with mugwort. You can never have too much mugwort! (+225 HP, Cure 1 Ailment).</t>
         </is>
       </c>
       <c r="G463" t="inlineStr">
@@ -18249,7 +18286,7 @@
       </c>
       <c r="F464" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 342. Restore debuffed stats.</t>
+          <t>An offering to a certain god (+342 HP, Clear Debuffs).</t>
         </is>
       </c>
       <c r="G464" t="inlineStr">
@@ -18289,7 +18326,7 @@
       </c>
       <c r="F465" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 38.</t>
+          <t>An inexpensive little cupful of cake (+38 HP).</t>
         </is>
       </c>
       <c r="G465" t="inlineStr">
@@ -18329,7 +18366,7 @@
       </c>
       <c r="F466" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100.</t>
+          <t>The perfect mid-afternoon snack. Loved by all (+100 HP).</t>
         </is>
       </c>
       <c r="G466" t="inlineStr">
@@ -18369,7 +18406,7 @@
       </c>
       <c r="F467" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200. Physical DEF +25%.</t>
+          <t>If you don't handle it with care, the cream will spurt all over you (+25% DEF).</t>
         </is>
       </c>
       <c r="G467" t="inlineStr">
@@ -18409,7 +18446,7 @@
       </c>
       <c r="F468" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 125.</t>
+          <t>Roll-shaped cake that people line up for ages to get (Party: +125 HP).</t>
         </is>
       </c>
       <c r="G468" t="inlineStr">
@@ -18449,7 +18486,7 @@
       </c>
       <c r="F469" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 180.</t>
+          <t>Triple-stack of pancakes smothered in sticky maple syrup (Party: +180 HP).</t>
         </is>
       </c>
       <c r="G469" t="inlineStr">
@@ -18489,7 +18526,7 @@
       </c>
       <c r="F470" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 300. Accuracy +25%.</t>
+          <t>It means white mountain. And yet, yellow cake. Y u do dis? (+300 HP).</t>
         </is>
       </c>
       <c r="G470" t="inlineStr">
@@ -18529,7 +18566,7 @@
       </c>
       <c r="F471" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 400. Evasion +25%.</t>
+          <t>Sweetness and justice are synonymous (+25% EVA).</t>
         </is>
       </c>
       <c r="G471" t="inlineStr">
@@ -18569,7 +18606,7 @@
       </c>
       <c r="F472" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 300.</t>
+          <t>A multi-layered, doughy pie cake (Party: +300 HP).</t>
         </is>
       </c>
       <c r="G472" t="inlineStr">
@@ -18609,7 +18646,7 @@
       </c>
       <c r="F473" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 200.</t>
+          <t>A luxury item perfect for souvenirs or gift exchanges (Party: +200 TP).</t>
         </is>
       </c>
       <c r="G473" t="inlineStr">
@@ -18649,7 +18686,7 @@
       </c>
       <c r="F474" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 60 and TP by 15.</t>
+          <t>Maple leaf-shaped souvenir confection. Even better as ice cream (+60 HP, +15 TP).</t>
         </is>
       </c>
       <c r="G474" t="inlineStr">
@@ -18689,7 +18726,7 @@
       </c>
       <c r="F475" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 125. May inflict Sleep (40%).</t>
+          <t>Liquor brewed from millet. Its mature flavor can become a habit (+125 HP, 40% Sleep).</t>
         </is>
       </c>
       <c r="G475" t="inlineStr">
@@ -18729,7 +18766,8 @@
       </c>
       <c r="F476" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 165. May inflict Blind (20%).</t>
+          <t>The mascot creature of this chocolate has yet to be identified by science.
+(+165 HP, 20% Blind)</t>
         </is>
       </c>
       <c r="G476" t="inlineStr">
@@ -18769,7 +18807,7 @@
       </c>
       <c r="F477" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200.</t>
+          <t>Canned whale. Slowly vanishing from shelves (+200 HP).</t>
         </is>
       </c>
       <c r="G477" t="inlineStr">
@@ -18809,7 +18847,7 @@
       </c>
       <c r="F478" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 240.</t>
+          <t>What you get when you toss a chunk of whale in your soup (Party: +240 HP).</t>
         </is>
       </c>
       <c r="G478" t="inlineStr">
@@ -18849,7 +18887,7 @@
       </c>
       <c r="F479" t="inlineStr">
         <is>
-          <t>Restore all allies' HP by 400.</t>
+          <t>Simple hotpot of whale and mizuna (Party: +400 HP).</t>
         </is>
       </c>
       <c r="G479" t="inlineStr">
@@ -18889,7 +18927,7 @@
       </c>
       <c r="F480" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 50.</t>
+          <t>Way too simple of a food. Really. It's just wheat (+50 HP).</t>
         </is>
       </c>
       <c r="G480" t="inlineStr">
@@ -18929,7 +18967,7 @@
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 120. Cure Freeze.</t>
+          <t>Filled with meat and veggies! Very delicious (+120 HP, Cure Freeze).</t>
         </is>
       </c>
       <c r="G481" t="inlineStr">
@@ -18969,7 +19007,7 @@
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 180. Cure Freeze.</t>
+          <t>Warms your body to the core on a cold day (+180 HP, Cure Freeze).</t>
         </is>
       </c>
       <c r="G482" t="inlineStr">
@@ -19009,7 +19047,7 @@
       </c>
       <c r="F483" t="inlineStr">
         <is>
-          <t>Speed DOWN -20%.</t>
+          <t>Jelly made with copious amounts of slime (Speed DOWN -20%.).</t>
         </is>
       </c>
       <c r="G483" t="inlineStr">
@@ -19049,7 +19087,7 @@
       </c>
       <c r="F484" t="inlineStr">
         <is>
-          <t>Speed DOWN -10%.</t>
+          <t>Made from only the gloopiest cuts of the slime (Speed DOWN -10%.).</t>
         </is>
       </c>
       <c r="G484" t="inlineStr">
@@ -19089,7 +19127,7 @@
       </c>
       <c r="F485" t="inlineStr">
         <is>
-          <t>Speed DOWN -40%.</t>
+          <t>So chewy it'll tire out your jaw (Speed DOWN -40%.).</t>
         </is>
       </c>
       <c r="G485" t="inlineStr">
@@ -19164,7 +19202,7 @@
       </c>
       <c r="F487" t="inlineStr">
         <is>
-          <t>Physical ATK +50%.</t>
+          <t>Spray that turns you into a super sadist for a few minutes (+50% ATK).</t>
         </is>
       </c>
       <c r="G487" t="inlineStr">
@@ -19199,7 +19237,7 @@
       </c>
       <c r="F488" t="inlineStr">
         <is>
-          <t>Physical ATK +75%. May inflict Blind (75%).</t>
+          <t>The feeling of being foreign. You're a stranger in a strange land (+75% ATK).</t>
         </is>
       </c>
       <c r="G488" t="inlineStr">
@@ -19239,7 +19277,8 @@
       </c>
       <c r="F489" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 150. Cure all status ailments.</t>
+          <t>Can stuffed with dragon meat. Rare and expensive but a little smelly.
+(+150 TP, Cure All Ailments)</t>
         </is>
       </c>
       <c r="G489" t="inlineStr">
@@ -19279,7 +19318,7 @@
       </c>
       <c r="F490" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 75. May inflict Sleep (30%).</t>
+          <t>No alcohol until you're 21! (+75 HP, 30% Sleep).</t>
         </is>
       </c>
       <c r="G490" t="inlineStr">
@@ -19319,7 +19358,8 @@
       </c>
       <c r="F491" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 150. May inflict Sleep (15%).</t>
+          <t>Some have never tried this sake, but none have tried it only once.
+(+150 HP, 15% Sleep)</t>
         </is>
       </c>
       <c r="G491" t="inlineStr">
@@ -19359,7 +19399,8 @@
       </c>
       <c r="F492" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 300. May inflict Blind (20%).</t>
+          <t>Powerful sake that intoxicates even heavy drinkers. Super harsh flavor.
+(+300 HP, 20% Blind)</t>
         </is>
       </c>
       <c r="G492" t="inlineStr">
@@ -19399,7 +19440,7 @@
       </c>
       <c r="F493" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 400. May inflict Sleep (20%).</t>
+          <t>Port wine carefully aged for over a hundred years (+400 HP, 20% Sleep).</t>
         </is>
       </c>
       <c r="G493" t="inlineStr">
@@ -19439,7 +19480,7 @@
       </c>
       <c r="F494" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 100.</t>
+          <t>Would you like some fries with that? (+100 HP/TP).</t>
         </is>
       </c>
       <c r="G494" t="inlineStr">
@@ -19479,7 +19520,7 @@
       </c>
       <c r="F495" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 150.</t>
+          <t>Taste aside, it's stiff and difficult to eat (+150 HP/TP).</t>
         </is>
       </c>
       <c r="G495" t="inlineStr">
@@ -19519,7 +19560,7 @@
       </c>
       <c r="F496" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 200. May inflict Paralysis (50%).</t>
+          <t>Dish made by shoving waterfowls into a dragon corpse (+200 HP/TP, 50% Paralysis).</t>
         </is>
       </c>
       <c r="G496" t="inlineStr">
@@ -19559,7 +19600,7 @@
       </c>
       <c r="F497" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 260. Evasion +25%.</t>
+          <t>A huge, hard egg. It's unbreakable (+25% EVA).</t>
         </is>
       </c>
       <c r="G497" t="inlineStr">
@@ -19599,7 +19640,7 @@
       </c>
       <c r="F498" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200 and TP by 50.</t>
+          <t>A snack so hard, you might chip a tooth when you bite into it (+200 HP, +50 TP).</t>
         </is>
       </c>
       <c r="G498" t="inlineStr">
@@ -19639,7 +19680,7 @@
       </c>
       <c r="F499" t="inlineStr">
         <is>
-          <t>Restore all allies' HP and TP by 200. Restore debuffed stats.</t>
+          <t>Cloying, syrupy drink (Party: +200 HP/TP, Clear Debuffs).</t>
         </is>
       </c>
       <c r="G499" t="inlineStr">
@@ -19679,7 +19720,7 @@
       </c>
       <c r="F500" t="inlineStr">
         <is>
-          <t>Inflict Poison (50% chance).</t>
+          <t>Meat so tender that it melts at the touch (50% Poison).</t>
         </is>
       </c>
       <c r="G500" t="inlineStr">
@@ -19719,7 +19760,7 @@
       </c>
       <c r="F501" t="inlineStr">
         <is>
-          <t>Inflict Poison (70% chance).</t>
+          <t>Meat is most delicious when it's almost rotten... or so they say (70% Poison).</t>
         </is>
       </c>
       <c r="G501" t="inlineStr">
@@ -19759,7 +19800,8 @@
       </c>
       <c r="F502" t="inlineStr">
         <is>
-          <t>Inflict Poison (95% chance). May inflict Paralysis (80%).</t>
+          <t>Primitive meat that shines suspiciously. Basically steroids in meat form.
+(95% Poison, 80% Paralysis)</t>
         </is>
       </c>
       <c r="G502" t="inlineStr">
@@ -19799,7 +19841,7 @@
       </c>
       <c r="F503" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 20.</t>
+          <t>Rich milk. I drink your 2% milk, Eli! I drink it up! (+20 HP/TP).</t>
         </is>
       </c>
       <c r="G503" t="inlineStr">
@@ -19839,7 +19881,7 @@
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100 and TP by 20.</t>
+          <t>Rich yogurt (+100 HP, +20 TP).</t>
         </is>
       </c>
       <c r="G504" t="inlineStr">
@@ -19879,7 +19921,7 @@
       </c>
       <c r="F505" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 200 and TP by 30.</t>
+          <t>Rich cheese (+200 HP, +30 TP).</t>
         </is>
       </c>
       <c r="G505" t="inlineStr">
@@ -19919,7 +19961,7 @@
       </c>
       <c r="F506" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 60.</t>
+          <t>Small candy with a rugged shape (Party: +60 TP).</t>
         </is>
       </c>
       <c r="G506" t="inlineStr">
@@ -19959,7 +20001,7 @@
       </c>
       <c r="F507" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 120. Cure Shadow Sew.</t>
+          <t>A larger-scale konpeito (Party: +120 TP, Cure Shadow Sew).</t>
         </is>
       </c>
       <c r="G507" t="inlineStr">
@@ -19999,7 +20041,7 @@
       </c>
       <c r="F508" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 400.</t>
+          <t>Konpeito as big as your fist (Party: +400 TP).</t>
         </is>
       </c>
       <c r="G508" t="inlineStr">
@@ -20039,7 +20081,7 @@
       </c>
       <c r="F509" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 100. May inflict Poison (40%).</t>
+          <t>Beverage squeezed out of an apple creature's insides (+100 HP/TP, 40% Poison).</t>
         </is>
       </c>
       <c r="G509" t="inlineStr">
@@ -20079,7 +20121,7 @@
       </c>
       <c r="F510" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 200. May inflict Poison (80%).</t>
+          <t>A candy with a whole appler trapped inside (+200 HP/TP, 80% Poison).</t>
         </is>
       </c>
       <c r="G510" t="inlineStr">
@@ -20119,7 +20161,7 @@
       </c>
       <c r="F511" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 100. May inflict Paralysis (90%).</t>
+          <t>Beverage squeezed out of a melon creature's insides (+100 HP/TP, 90% Paralysis).</t>
         </is>
       </c>
       <c r="G511" t="inlineStr">
@@ -20159,7 +20201,8 @@
       </c>
       <c r="F512" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 200. May inflict Paralysis (80%).</t>
+          <t>Unrelated to that anime character who lets people eat her face.
+(+200 HP/TP, 80% Paralysis)</t>
         </is>
       </c>
       <c r="G512" t="inlineStr">
@@ -20199,7 +20242,7 @@
       </c>
       <c r="F513" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 100. May inflict Silence (40%).</t>
+          <t>Beverage squeezed out of a banana creature's insides (+100 HP/TP, 40% Silence).</t>
         </is>
       </c>
       <c r="G513" t="inlineStr">
@@ -20239,7 +20282,7 @@
       </c>
       <c r="F514" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 200. May inflict Silence (80%).</t>
+          <t>It's a big banana. Looks pretty sexy (+200 HP/TP, 80% Silence).</t>
         </is>
       </c>
       <c r="G514" t="inlineStr">
@@ -20279,7 +20322,7 @@
       </c>
       <c r="F515" t="inlineStr">
         <is>
-          <t>Inflict Blind (10% chance).</t>
+          <t>A Fairy Mandra that's badly wounded (10% Blind).</t>
         </is>
       </c>
       <c r="G515" t="inlineStr">
@@ -20319,7 +20362,7 @@
       </c>
       <c r="F516" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 160.</t>
+          <t>Best when stuck on a skewer and grilled (+160 HP).</t>
         </is>
       </c>
       <c r="G516" t="inlineStr">
@@ -20359,7 +20402,7 @@
       </c>
       <c r="F517" t="inlineStr">
         <is>
-          <t>Cure all status ailments for an ally.</t>
+          <t>Can be used as herbal medicine. It has a strong scent (Cure All Ailments).</t>
         </is>
       </c>
       <c r="G517" t="inlineStr">
@@ -20399,7 +20442,7 @@
       </c>
       <c r="F518" t="inlineStr">
         <is>
-          <t>Restore all allies' TP by 150.</t>
+          <t>The trefoil of a mandra, used as a graduation charm (Party: +150 TP).</t>
         </is>
       </c>
       <c r="G518" t="inlineStr">
@@ -20439,7 +20482,7 @@
       </c>
       <c r="F519" t="inlineStr">
         <is>
-          <t>Inflict Silence (95% chance). May inflict Freeze (95%).</t>
+          <t>Made by grinding up mandras (95% Silence, 95% Freeze).</t>
         </is>
       </c>
       <c r="G519" t="inlineStr">
@@ -20479,7 +20522,7 @@
       </c>
       <c r="F520" t="inlineStr">
         <is>
-          <t>Inflict Poison (15% chance).</t>
+          <t>An Otherworld Mandra that's badly wounded (15% Poison).</t>
         </is>
       </c>
       <c r="G520" t="inlineStr">
@@ -20519,7 +20562,7 @@
       </c>
       <c r="F521" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 80.</t>
+          <t>Slice it thin and eat it like sashimi (+80 TP).</t>
         </is>
       </c>
       <c r="G521" t="inlineStr">
@@ -20559,7 +20602,7 @@
       </c>
       <c r="F522" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 350. Cure Shadow Sew.</t>
+          <t>Goes really well with meat rolls (+350 HP, Cure Shadow Sew).</t>
         </is>
       </c>
       <c r="G522" t="inlineStr">
@@ -20634,7 +20677,7 @@
       </c>
       <c r="F524" t="inlineStr">
         <is>
-          <t>Restore all allies' HP and TP by 2,000.</t>
+          <t>Freshly squeezed mandra juice. Nice and pulpy (Party: +2000 HP/TP).</t>
         </is>
       </c>
       <c r="G524" t="inlineStr">
@@ -20674,7 +20717,7 @@
       </c>
       <c r="F525" t="inlineStr">
         <is>
-          <t>Restore all allies' HP and TP by 1,000.</t>
+          <t>Said to bring good fortune. Does anyone actually believe that? (Party: +1000 HP/TP).</t>
         </is>
       </c>
       <c r="G525" t="inlineStr">
@@ -20714,7 +20757,7 @@
       </c>
       <c r="F526" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 7.</t>
+          <t>Freshly squeezed, straight from OC (+7 HP/TP).</t>
         </is>
       </c>
       <c r="G526" t="inlineStr">
@@ -20754,7 +20797,7 @@
       </c>
       <c r="F527" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 14.</t>
+          <t>Strange rice cooked with tangerine juice (+14 HP/TP).</t>
         </is>
       </c>
       <c r="G527" t="inlineStr">
@@ -20794,7 +20837,7 @@
       </c>
       <c r="F528" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 45.</t>
+          <t>A cafe au lait mixed with oranges. It's scalding hot (+45 HP/TP).</t>
         </is>
       </c>
       <c r="G528" t="inlineStr">
@@ -20834,7 +20877,7 @@
       </c>
       <c r="F529" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 13.</t>
+          <t>Full of vitamins. Have some after you exercise (+13 HP/TP).</t>
         </is>
       </c>
       <c r="G529" t="inlineStr">
@@ -20874,7 +20917,7 @@
       </c>
       <c r="F530" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 22.</t>
+          <t>Sweet pie that's made with tons of cherries (+22 HP/TP).</t>
         </is>
       </c>
       <c r="G530" t="inlineStr">
@@ -20914,7 +20957,8 @@
       </c>
       <c r="F531" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 50. Cure all status ailments.</t>
+          <t>Made in an attempt to achieve sake supremacy. To sake-cceed.
+(+50 HP/TP, Cure All Ailments)</t>
         </is>
       </c>
       <c r="G531" t="inlineStr">
@@ -20954,7 +20998,7 @@
       </c>
       <c r="F532" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 1,000.</t>
+          <t>The denizens of the world above say these pair well with tea (+1000 TP).</t>
         </is>
       </c>
       <c r="G532" t="inlineStr">
@@ -20994,7 +21038,7 @@
       </c>
       <c r="F533" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 65.</t>
+          <t>Moon cake with just the right level of sweetness (+65 TP).</t>
         </is>
       </c>
       <c r="G533" t="inlineStr">
@@ -21034,7 +21078,7 @@
       </c>
       <c r="F534" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 130.</t>
+          <t>Rice cake that crumbles from the outside as you eat it (+130 TP).</t>
         </is>
       </c>
       <c r="G534" t="inlineStr">
@@ -21074,7 +21118,8 @@
       </c>
       <c r="F535" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 999. Cure all status ailments.</t>
+          <t>Precious, sweet-smelling beverage made of liquified mana crystals.
+(+999 TP, Cure All Ailments)</t>
         </is>
       </c>
       <c r="G535" t="inlineStr">
@@ -21114,7 +21159,7 @@
       </c>
       <c r="F536" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 5,000.</t>
+          <t>Dangerous drink that lights a fire in your loins. Yowch! That's hot! (+5000 HP).</t>
         </is>
       </c>
       <c r="G536" t="inlineStr">
@@ -21154,7 +21199,7 @@
       </c>
       <c r="F537" t="inlineStr">
         <is>
-          <t>Permanently grant +9 Skill Points (SP) to an ally.</t>
+          <t>Stained with the blood of sacrifice. It's golden underneath (+9 SP).</t>
         </is>
       </c>
       <c r="G537" t="inlineStr">
@@ -21194,7 +21239,7 @@
       </c>
       <c r="F538" t="inlineStr">
         <is>
-          <t>Cure Freeze for an ally.</t>
+          <t>The most treasured treasure of the Dragon Palace... cures Freeze (Cure Freeze).</t>
         </is>
       </c>
       <c r="G538" t="inlineStr">
@@ -21269,7 +21314,7 @@
       </c>
       <c r="F540" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 1,000 and clear stat debuffs.</t>
+          <t>A magical egg. There's a whole new world inside it (+1000 HP, Clear Debuffs).</t>
         </is>
       </c>
       <c r="G540" t="inlineStr">
@@ -21309,7 +21354,7 @@
       </c>
       <c r="F541" t="inlineStr">
         <is>
-          <t>Instantly escape from the dungeon back to base.</t>
+          <t>Proof that you've attended all of Miss Euthys's lectures (Escape Dungeon).</t>
         </is>
       </c>
       <c r="G541" t="inlineStr">
@@ -21349,7 +21394,7 @@
       </c>
       <c r="F542" t="inlineStr">
         <is>
-          <t>Restore an ally's TP by 50.</t>
+          <t>A fruit from the garden of Paradise (+50 TP).</t>
         </is>
       </c>
       <c r="G542" t="inlineStr">
@@ -21389,7 +21434,7 @@
       </c>
       <c r="F543" t="inlineStr">
         <is>
-          <t>Cure all status ailments for an ally.</t>
+          <t>Huskin' makes me feel good (Cure All Ailments).</t>
         </is>
       </c>
       <c r="G543" t="inlineStr">
@@ -21429,7 +21474,7 @@
       </c>
       <c r="F544" t="inlineStr">
         <is>
-          <t>Restore an ally's HP by 100.</t>
+          <t>The original underlying form of all matter in the universe (+100 HP).</t>
         </is>
       </c>
       <c r="G544" t="inlineStr">
@@ -21469,7 +21514,7 @@
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>Restore an ally's HP and TP by 10.</t>
+          <t>Dry and dead. It won't grow into anything more (+10 HP/TP).</t>
         </is>
       </c>
       <c r="G545" t="inlineStr">
@@ -21509,7 +21554,7 @@
       </c>
       <c r="F546" t="inlineStr">
         <is>
-          <t>Inflict Silence (95% chance).</t>
+          <t>A precious book depicting powerful bonds between men (95% Silence).</t>
         </is>
       </c>
       <c r="G546" t="inlineStr">

</xml_diff>